<commit_message>
feat: add Power BI executive reporting pack
</commit_message>
<xml_diff>
--- a/excel/Helio_SaaS_FP&A_Operating_Model.xlsx
+++ b/excel/Helio_SaaS_FP&A_Operating_Model.xlsx
@@ -5749,7 +5749,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -6630,7 +6630,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="C30" s="32" t="inlineStr">
         <is>
-          <t>2026-08-25 06:04 UTC</t>
+          <t>2026-08-27 05:16 UTC</t>
         </is>
       </c>
       <c r="E30" s="128" t="inlineStr">
@@ -9603,7 +9603,7 @@
         <v>254568</v>
       </c>
       <c r="G30" s="48" t="n">
-        <v>339460.6800000001</v>
+        <v>339460.6799999999</v>
       </c>
       <c r="H30" s="48" t="n">
         <v>2107.44</v>
@@ -9615,7 +9615,7 @@
         <v>-197466.12</v>
       </c>
       <c r="K30" s="48" t="n">
-        <v>325583.88</v>
+        <v>325583.8799999999</v>
       </c>
       <c r="L30" s="48" t="n">
         <v>27793280.76</v>
@@ -10304,7 +10304,7 @@
         <v>29388435.72</v>
       </c>
       <c r="F46" s="48" t="n">
-        <v>815749.3199999999</v>
+        <v>815749.3200000001</v>
       </c>
       <c r="G46" s="48" t="n">
         <v>245648.28</v>
@@ -10319,7 +10319,7 @@
         <v>-220801.08</v>
       </c>
       <c r="K46" s="48" t="n">
-        <v>800880.12</v>
+        <v>800880.1200000002</v>
       </c>
       <c r="L46" s="48" t="n">
         <v>30189315.84</v>
@@ -11360,7 +11360,7 @@
         <v>32493210.36</v>
       </c>
       <c r="F70" s="48" t="n">
-        <v>650292.3600000001</v>
+        <v>650292.36</v>
       </c>
       <c r="G70" s="48" t="n">
         <v>510603.96</v>
@@ -23992,7 +23992,7 @@
         <v>33553421.70294353</v>
       </c>
       <c r="C2" s="48" t="n">
-        <v>32571935.84232378</v>
+        <v>32571935.84232377</v>
       </c>
       <c r="D2" s="48" t="n">
         <v>-5910400.124143494</v>
@@ -24205,7 +24205,7 @@
         </is>
       </c>
       <c r="B4" s="48" t="n">
-        <v>36123036.63015183</v>
+        <v>36123036.63015182</v>
       </c>
       <c r="C4" s="48" t="n">
         <v>33024317.95014933</v>
@@ -24214,7 +24214,7 @@
         <v>-5507025.088939572</v>
       </c>
       <c r="E4" s="48" t="n">
-        <v>46032954.52691904</v>
+        <v>46032954.52691905</v>
       </c>
       <c r="F4" s="48" t="n">
         <v>18953992.75157869</v>
@@ -24516,7 +24516,7 @@
         </is>
       </c>
       <c r="U9" s="48" t="n">
-        <v>33655579.61198956</v>
+        <v>33655579.61198955</v>
       </c>
       <c r="V9" s="48" t="n">
         <v>33985619.40904452</v>
@@ -24622,7 +24622,7 @@
         </is>
       </c>
       <c r="U11" s="48" t="n">
-        <v>33767560.74630731</v>
+        <v>33767560.74630732</v>
       </c>
       <c r="V11" s="48" t="n">
         <v>34388015.77012163</v>
@@ -24722,7 +24722,7 @@
         <v>34816416.56479766</v>
       </c>
       <c r="W13" s="48" t="n">
-        <v>36123036.63015183</v>
+        <v>36123036.63015182</v>
       </c>
       <c r="Z13" s="19" t="inlineStr">
         <is>
@@ -24769,7 +24769,7 @@
         <v>34980843.62572146</v>
       </c>
       <c r="W14" s="48" t="n">
-        <v>36615401.63381294</v>
+        <v>36615401.63381295</v>
       </c>
       <c r="Z14" s="19" t="inlineStr">
         <is>
@@ -24951,13 +24951,13 @@
         </is>
       </c>
       <c r="U18" s="48" t="n">
-        <v>34174814.84644881</v>
+        <v>34174814.8464488</v>
       </c>
       <c r="V18" s="48" t="n">
         <v>36829763.61356527</v>
       </c>
       <c r="W18" s="48" t="n">
-        <v>39588967.34456072</v>
+        <v>39588967.34456073</v>
       </c>
       <c r="Z18" s="19" t="inlineStr">
         <is>
@@ -25051,13 +25051,13 @@
         </is>
       </c>
       <c r="U20" s="48" t="n">
-        <v>34766211.13177589</v>
+        <v>34766211.1317759</v>
       </c>
       <c r="V20" s="48" t="n">
         <v>37904852.39349368</v>
       </c>
       <c r="W20" s="48" t="n">
-        <v>41199683.08172435</v>
+        <v>41199683.08172434</v>
       </c>
       <c r="Z20" s="19" t="inlineStr">
         <is>
@@ -25304,7 +25304,7 @@
         <v>41566296.05586515</v>
       </c>
       <c r="W25" s="48" t="n">
-        <v>46032954.52691904</v>
+        <v>46032954.52691905</v>
       </c>
       <c r="Z25" s="19" t="inlineStr">
         <is>
@@ -26137,16 +26137,16 @@
         <v>2920858.782250161</v>
       </c>
       <c r="P3" s="48" t="n">
-        <v>850000.0000000003</v>
+        <v>850000</v>
       </c>
       <c r="Q3" s="118" t="n">
-        <v>25.6470588235294</v>
+        <v>25.64705882352941</v>
       </c>
       <c r="R3" s="118" t="n">
         <v>24</v>
       </c>
       <c r="S3" s="109" t="n">
-        <v>1.647058823529402</v>
+        <v>1.647058823529413</v>
       </c>
       <c r="T3" s="19" t="inlineStr">
         <is>
@@ -26160,13 +26160,13 @@
         <v>0</v>
       </c>
       <c r="W3" s="48" t="n">
-        <v>-3.725290298461914e-09</v>
+        <v>0</v>
       </c>
       <c r="X3" s="48" t="n">
-        <v>-7.450580596923828e-09</v>
+        <v>0</v>
       </c>
       <c r="Y3" s="48" t="n">
-        <v>-3.725290298461914e-09</v>
+        <v>0</v>
       </c>
       <c r="Z3" s="19" t="inlineStr">
         <is>
@@ -26227,7 +26227,7 @@
         <v>2996583.27052319</v>
       </c>
       <c r="P4" s="48" t="n">
-        <v>883984.7124660934</v>
+        <v>883984.7124660932</v>
       </c>
       <c r="Q4" s="118" t="n">
         <v>24.66105996243252</v>
@@ -26236,7 +26236,7 @@
         <v>24</v>
       </c>
       <c r="S4" s="109" t="n">
-        <v>0.6610599624325211</v>
+        <v>0.6610599624325246</v>
       </c>
       <c r="T4" s="19" t="inlineStr">
         <is>
@@ -26250,7 +26250,7 @@
         <v>-31366.64182941336</v>
       </c>
       <c r="W4" s="48" t="n">
-        <v>-637083.11137514</v>
+        <v>-637083.1113751382</v>
       </c>
       <c r="X4" s="48" t="n">
         <v>466.8747128918767</v>
@@ -26281,19 +26281,19 @@
         </is>
       </c>
       <c r="D5" s="48" t="n">
-        <v>850000.0000000003</v>
+        <v>850000</v>
       </c>
       <c r="E5" s="48" t="n">
         <v>21800000</v>
       </c>
       <c r="F5" s="118" t="n">
-        <v>25.6470588235294</v>
+        <v>25.64705882352941</v>
       </c>
       <c r="G5" s="118" t="n">
         <v>24</v>
       </c>
       <c r="H5" s="109" t="n">
-        <v>1.647058823529402</v>
+        <v>1.647058823529413</v>
       </c>
       <c r="I5" s="19" t="inlineStr">
         <is>
@@ -26318,7 +26318,7 @@
         </is>
       </c>
       <c r="D6" s="48" t="n">
-        <v>883984.7124660934</v>
+        <v>883984.7124660932</v>
       </c>
       <c r="E6" s="48" t="n">
         <v>21800000</v>
@@ -26330,7 +26330,7 @@
         <v>24</v>
       </c>
       <c r="H6" s="109" t="n">
-        <v>0.6610599624325211</v>
+        <v>0.6610599624325246</v>
       </c>
       <c r="I6" s="19" t="inlineStr">
         <is>
@@ -26588,7 +26588,7 @@
         </is>
       </c>
       <c r="L2" s="48" t="n">
-        <v>5256937.089999999</v>
+        <v>5256937.09</v>
       </c>
       <c r="M2" s="48" t="n">
         <v>6718668.05</v>
@@ -26699,13 +26699,13 @@
         <v>7135686.970000001</v>
       </c>
       <c r="M3" s="48" t="n">
-        <v>5136850.399999999</v>
+        <v>5136850.4</v>
       </c>
       <c r="N3" s="48" t="n">
         <v>5254093.74</v>
       </c>
       <c r="O3" s="48" t="n">
-        <v>2095.259999999981</v>
+        <v>2095.25999999998</v>
       </c>
       <c r="P3" s="48" t="n">
         <v>7020538.889999998</v>
@@ -26714,7 +26714,7 @@
         <v>220789.2500000001</v>
       </c>
       <c r="R3" s="124" t="n">
-        <v>-1.862645149230957e-09</v>
+        <v>-2.793967723846436e-09</v>
       </c>
       <c r="U3" s="19" t="inlineStr">
         <is>
@@ -26886,13 +26886,13 @@
         <v>6029572.379999998</v>
       </c>
       <c r="M5" s="48" t="n">
-        <v>6523735.300000001</v>
+        <v>6523735.3</v>
       </c>
       <c r="N5" s="48" t="n">
         <v>5879791.560000001</v>
       </c>
       <c r="O5" s="48" t="n">
-        <v>23987.41000000003</v>
+        <v>23987.41000000006</v>
       </c>
       <c r="P5" s="48" t="n">
         <v>6697503.529999999</v>
@@ -26954,7 +26954,7 @@
         <v>6310786.96</v>
       </c>
       <c r="O6" s="48" t="n">
-        <v>13269.76999999967</v>
+        <v>13269.76999999964</v>
       </c>
       <c r="P6" s="48" t="n">
         <v>8622826.389999999</v>
@@ -27100,7 +27100,7 @@
         <v>7633041.97</v>
       </c>
       <c r="O10" s="48" t="n">
-        <v>7109.839999999676</v>
+        <v>7109.839999999735</v>
       </c>
       <c r="P10" s="48" t="n">
         <v>11557796.34</v>
@@ -27128,7 +27128,7 @@
         <v>8079773.71</v>
       </c>
       <c r="O11" s="48" t="n">
-        <v>17865.61000000045</v>
+        <v>17865.61000000034</v>
       </c>
       <c r="P11" s="48" t="n">
         <v>10563773.5</v>
@@ -27137,7 +27137,7 @@
         <v>325963.7100000005</v>
       </c>
       <c r="R11" s="124" t="n">
-        <v>0</v>
+        <v>1.862645149230957e-09</v>
       </c>
     </row>
   </sheetData>
@@ -27207,7 +27207,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -27557,7 +27557,7 @@
         <v>254568</v>
       </c>
       <c r="F18" s="40" t="n">
-        <v>339460.6800000001</v>
+        <v>339460.6799999999</v>
       </c>
       <c r="G18" s="40" t="n">
         <v>2107.44</v>
@@ -27686,7 +27686,7 @@
         <v>29388435.72</v>
       </c>
       <c r="E22" s="40" t="n">
-        <v>815749.3199999999</v>
+        <v>815749.3200000001</v>
       </c>
       <c r="F22" s="40" t="n">
         <v>245648.28</v>
@@ -27884,7 +27884,7 @@
         <v>32493210.36</v>
       </c>
       <c r="E28" s="40" t="n">
-        <v>650292.3600000001</v>
+        <v>650292.36</v>
       </c>
       <c r="F28" s="40" t="n">
         <v>510603.96</v>
@@ -29841,7 +29841,7 @@
         </is>
       </c>
       <c r="B52" s="48" t="n">
-        <v>36123036.63015183</v>
+        <v>36123036.63015182</v>
       </c>
     </row>
     <row r="55">
@@ -30109,7 +30109,7 @@
         <v>254568</v>
       </c>
       <c r="C70" s="48" t="n">
-        <v>339460.6800000001</v>
+        <v>339460.6799999999</v>
       </c>
       <c r="D70" s="48" t="n">
         <v>2107.44</v>
@@ -30194,7 +30194,7 @@
         </is>
       </c>
       <c r="B74" s="48" t="n">
-        <v>815749.3199999999</v>
+        <v>815749.3200000001</v>
       </c>
       <c r="C74" s="48" t="n">
         <v>245648.28</v>
@@ -30326,7 +30326,7 @@
         </is>
       </c>
       <c r="B80" s="48" t="n">
-        <v>650292.3600000001</v>
+        <v>650292.36</v>
       </c>
       <c r="C80" s="48" t="n">
         <v>510603.96</v>
@@ -30684,7 +30684,7 @@
         </is>
       </c>
       <c r="B103" s="48" t="n">
-        <v>33655579.61198956</v>
+        <v>33655579.61198955</v>
       </c>
       <c r="C103" s="48" t="n">
         <v>33985619.40904452</v>
@@ -30716,7 +30716,7 @@
         </is>
       </c>
       <c r="B105" s="48" t="n">
-        <v>33767560.74630731</v>
+        <v>33767560.74630732</v>
       </c>
       <c r="C105" s="48" t="n">
         <v>34388015.77012163</v>
@@ -30754,7 +30754,7 @@
         <v>34816416.56479766</v>
       </c>
       <c r="D107" s="48" t="n">
-        <v>36123036.63015183</v>
+        <v>36123036.63015182</v>
       </c>
     </row>
     <row r="108">
@@ -30770,7 +30770,7 @@
         <v>34980843.62572146</v>
       </c>
       <c r="D108" s="48" t="n">
-        <v>36615401.63381294</v>
+        <v>36615401.63381295</v>
       </c>
     </row>
     <row r="109">
@@ -30828,13 +30828,13 @@
         </is>
       </c>
       <c r="B112" s="48" t="n">
-        <v>34174814.84644881</v>
+        <v>34174814.8464488</v>
       </c>
       <c r="C112" s="48" t="n">
         <v>36829763.61356527</v>
       </c>
       <c r="D112" s="48" t="n">
-        <v>39588967.34456072</v>
+        <v>39588967.34456073</v>
       </c>
     </row>
     <row r="113">
@@ -30860,13 +30860,13 @@
         </is>
       </c>
       <c r="B114" s="48" t="n">
-        <v>34766211.13177589</v>
+        <v>34766211.1317759</v>
       </c>
       <c r="C114" s="48" t="n">
         <v>37904852.39349368</v>
       </c>
       <c r="D114" s="48" t="n">
-        <v>41199683.08172435</v>
+        <v>41199683.08172434</v>
       </c>
     </row>
     <row r="115">
@@ -30946,7 +30946,7 @@
         <v>41566296.05586515</v>
       </c>
       <c r="D119" s="48" t="n">
-        <v>46032954.52691904</v>
+        <v>46032954.52691905</v>
       </c>
     </row>
     <row r="122">
@@ -30989,7 +30989,7 @@
         <v>0</v>
       </c>
       <c r="C124" s="48" t="n">
-        <v>-3.725290298461914e-09</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="125">
@@ -31002,7 +31002,7 @@
         <v>147322.040569365</v>
       </c>
       <c r="C125" s="48" t="n">
-        <v>-637083.11137514</v>
+        <v>-637083.1113751382</v>
       </c>
     </row>
   </sheetData>
@@ -31062,7 +31062,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -32107,7 +32107,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -32334,7 +32334,7 @@
         <v>170863.2</v>
       </c>
       <c r="I11" s="72" t="n">
-        <v>650292.3600000001</v>
+        <v>650292.36</v>
       </c>
       <c r="J11" s="73" t="n">
         <v>379723.8431657766</v>
@@ -33571,7 +33571,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -34480,7 +34480,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -35524,7 +35524,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -36172,7 +36172,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -36753,13 +36753,13 @@
         </is>
       </c>
       <c r="D49" s="54" t="n">
-        <v>850000.0000000003</v>
+        <v>850000</v>
       </c>
       <c r="E49" s="114" t="n">
-        <v>25.6470588235294</v>
+        <v>25.64705882352941</v>
       </c>
       <c r="F49" s="109" t="n">
-        <v>1.647058823529402</v>
+        <v>1.647058823529413</v>
       </c>
       <c r="G49" s="24" t="inlineStr">
         <is>
@@ -36779,13 +36779,13 @@
         </is>
       </c>
       <c r="D50" s="54" t="n">
-        <v>883984.7124660934</v>
+        <v>883984.7124660932</v>
       </c>
       <c r="E50" s="114" t="n">
         <v>24.66105996243252</v>
       </c>
       <c r="F50" s="109" t="n">
-        <v>0.6610599624325211</v>
+        <v>0.6610599624325246</v>
       </c>
       <c r="G50" s="24" t="inlineStr">
         <is>
@@ -36888,7 +36888,7 @@
     <row r="4" ht="11.5" customHeight="1">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Workbook v1.0  |  built 2026-08-25 06:04 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
+          <t>Workbook v1.0  |  built 2026-08-27 05:16 UTC  |  source: data/marts (Phase 3-8 analytical layer, frozen)</t>
         </is>
       </c>
     </row>
@@ -37205,7 +37205,7 @@
         </is>
       </c>
       <c r="C31" s="48" t="n">
-        <v>5256937.089999999</v>
+        <v>5256937.09</v>
       </c>
       <c r="D31" s="48" t="n">
         <v>6718668.05</v>
@@ -37237,13 +37237,13 @@
         <v>7135686.970000001</v>
       </c>
       <c r="D32" s="48" t="n">
-        <v>5136850.399999999</v>
+        <v>5136850.4</v>
       </c>
       <c r="E32" s="48" t="n">
         <v>5254093.74</v>
       </c>
       <c r="F32" s="48" t="n">
-        <v>2095.259999999981</v>
+        <v>2095.25999999998</v>
       </c>
       <c r="G32" s="122" t="n">
         <v>7020538.889999998</v>
@@ -37295,13 +37295,13 @@
         <v>6029572.379999998</v>
       </c>
       <c r="D34" s="48" t="n">
-        <v>6523735.300000001</v>
+        <v>6523735.3</v>
       </c>
       <c r="E34" s="48" t="n">
         <v>5879791.560000001</v>
       </c>
       <c r="F34" s="48" t="n">
-        <v>23987.41000000003</v>
+        <v>23987.41000000006</v>
       </c>
       <c r="G34" s="122" t="n">
         <v>6697503.529999999</v>
@@ -37330,7 +37330,7 @@
         <v>6310786.96</v>
       </c>
       <c r="F35" s="48" t="n">
-        <v>13269.76999999967</v>
+        <v>13269.76999999964</v>
       </c>
       <c r="G35" s="122" t="n">
         <v>8622826.389999999</v>
@@ -37446,7 +37446,7 @@
         <v>7633041.97</v>
       </c>
       <c r="F39" s="48" t="n">
-        <v>7109.839999999676</v>
+        <v>7109.839999999735</v>
       </c>
       <c r="G39" s="122" t="n">
         <v>11557796.34</v>
@@ -37475,7 +37475,7 @@
         <v>8079773.71</v>
       </c>
       <c r="F40" s="48" t="n">
-        <v>17865.61000000045</v>
+        <v>17865.61000000034</v>
       </c>
       <c r="G40" s="122" t="n">
         <v>10563773.5</v>

</xml_diff>